<commit_message>
docs: ajusta equipe para 3 devs (Max, Lucas, Lorenzo) e adiciona Unisinos
- Substitui composição de 'Par A + Par B' (4 devs) pelo modelo 'Par + Solo'
  com rotação semanal entre 3 devs: Max Soares, Lucas Mendes, Lorenzo Oliveira
- Adiciona referência à Universidade do Vale do Rio dos Sinos (Unisinos) na
  capa do Plano de Projeto, README e atas
- Recalcula esforço por desenvolvedor na planilha UCP: 368 h/dev total e
  ~74 h/semana por dev (Carga semanal — alerta passou a indicar 'Acima do
  recomendado'); adiciona risco R5b 'Carga semanal alta com 3 devs'
- Atualiza Plano de Projeto §4 com tabela de rotação par + solo das sprints
  1 a 4 e Plano de Projeto §11 com 'par + solo' no lugar de 'Par A + Par B'
- Atualiza Checklist_Sprint1.xlsx com responsáveis nomeados (Max, Lucas,
  Lorenzo, Equipe) e marca itens já entregues nesta primeira semana
- Atualiza atas review, retro e trello para refletir os três membros, com
  Lorenzo Oliveira como Scrum Master e Lucas Mendes como owner do repo
</commit_message>
<xml_diff>
--- a/docs/Checklist_Sprint1.xlsx
+++ b/docs/Checklist_Sprint1.xlsx
@@ -25,9 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="175">
-  <si>
-    <t xml:space="preserve">MANGO — CHECKLIST DA SPRINT 1 (Entrega 1: Planejamento e Estruturação)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="175">
+  <si>
+    <t xml:space="preserve">MANGO — CHECKLIST DA SPRINT 1 · Unisinos 2026/1 (Entrega 1: Planejamento e Estruturação)</t>
   </si>
   <si>
     <t xml:space="preserve">22 itens distribuídos em 4 critérios (Produto 4 · Processo 7 · Config. Software 8 · Qualidade 3). Atualize Status semanalmente.</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Board Trello</t>
   </si>
   <si>
-    <t xml:space="preserve">[def]</t>
+    <t xml:space="preserve">Lorenzo</t>
   </si>
   <si>
     <t xml:space="preserve">URL do board</t>
@@ -171,9 +171,6 @@
     <t xml:space="preserve">Ata de Planning</t>
   </si>
   <si>
-    <t xml:space="preserve">Scrum M.</t>
-  </si>
-  <si>
     <t xml:space="preserve">docs/atas/planning-sprint1.md</t>
   </si>
   <si>
@@ -189,6 +186,9 @@
     <t xml:space="preserve">docs/atas/dailies-sprint1.md</t>
   </si>
   <si>
+    <t xml:space="preserve">Em Andamento</t>
+  </si>
+  <si>
     <t xml:space="preserve">Realizar a Revisão da Sprint (apresentar entregas).</t>
   </si>
   <si>
@@ -219,7 +219,10 @@
     <t xml:space="preserve">Repo + URL</t>
   </si>
   <si>
-    <t xml:space="preserve">URL do repo</t>
+    <t xml:space="preserve">Lucas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">github.com/lucsmends/mango.dev</t>
   </si>
   <si>
     <t xml:space="preserve">Configurar o GitFlow: criar branches main e develop.</t>
@@ -291,7 +294,7 @@
     <t xml:space="preserve">.gitignore na raiz</t>
   </si>
   <si>
-    <t xml:space="preserve">Fazer commit inicial e push de cada membro do time (4 devs).</t>
+    <t xml:space="preserve">Fazer commit inicial e push de cada membro do time (3 devs).</t>
   </si>
   <si>
     <t xml:space="preserve">Git · Commits</t>
@@ -333,7 +336,7 @@
     <t xml:space="preserve">Checklist_Sprint1.xlsx (este arquivo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Revisão cruzada: Par B valida artefatos do Par A (e vice-versa).</t>
+    <t xml:space="preserve">Revisão cruzada: Solo valida artefatos do Par (e vice-versa).</t>
   </si>
   <si>
     <t xml:space="preserve">Revisão · Pares</t>
@@ -342,9 +345,6 @@
     <t xml:space="preserve">Evidência de revisão</t>
   </si>
   <si>
-    <t xml:space="preserve">Pares</t>
-  </si>
-  <si>
     <t xml:space="preserve">docs/atas/revisao-cruzada-sprint1.md</t>
   </si>
   <si>
@@ -378,9 +378,6 @@
     <t xml:space="preserve">Artefato pronto, validado e linkado na coluna Evidência.</t>
   </si>
   <si>
-    <t xml:space="preserve">Em Andamento</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pessoa responsável trabalhando ativamente na tarefa.</t>
   </si>
   <si>
@@ -432,58 +429,61 @@
     <t xml:space="preserve">E-mail / GitHub</t>
   </si>
   <si>
+    <t xml:space="preserve">Função na sprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint focal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev · Product Owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Soares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max.ho.soares@gmail.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Par</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint focal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product Owner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Ho Soares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max.ho.soares@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Par A</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sprint 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Scrum Master</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[a definir]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev (Par A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev (Par B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Par B</t>
+    <t xml:space="preserve">Dev · Owner do repo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucas Mendes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lucsmends (GitHub)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev · Scrum Master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorenzo Oliveira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo</t>
   </si>
   <si>
     <t xml:space="preserve">Rotação de pares</t>
   </si>
   <si>
-    <t xml:space="preserve">• Sprint 1: composição inicial (acima).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 2: troca de 1 membro entre os pares.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 3: nova rotação para garantir que todos passem por todos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 4: composição que dê suporte ao desafio do UC4 (OCR/tradução).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Cada par desenvolve uma 'fatia vertical' do UC da semana (Banco → Service → Controller).</t>
+    <t xml:space="preserve">• Sprint 1: Par = Max + Lucas · Solo = Lorenzo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 2: Par = Lucas + Lorenzo · Solo = Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 3: Par = Max + Lorenzo · Solo = Lucas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4: Par = Max + Lucas · Solo = Lorenzo (volta à composição da Sprint 1 para o desafio do UC4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O par desenvolve a fatia vertical principal do UC; o solo cobre fatia complementar e revisa o PR cruzado.</t>
   </si>
   <si>
     <t xml:space="preserve">SPRINT 1 — META E DEFINIÇÕES</t>
@@ -1438,13 +1438,13 @@
         <v>47</v>
       </c>
       <c r="F12" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="12" t="s">
-        <v>49</v>
-      </c>
       <c r="H12" s="8" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1455,22 +1455,22 @@
         <v>29</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>14</v>
       </c>
       <c r="G13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1516,7 +1516,7 @@
         <v>58</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>59</v>
@@ -1542,13 +1542,13 @@
         <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1559,22 +1559,22 @@
         <v>60</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1585,19 +1585,19 @@
         <v>60</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>14</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>16</v>
@@ -1611,19 +1611,19 @@
         <v>60</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>16</v>
@@ -1637,22 +1637,22 @@
         <v>60</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>42</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,19 +1663,19 @@
         <v>60</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>16</v>
@@ -1689,22 +1689,22 @@
         <v>60</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>42</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,22 +1715,22 @@
         <v>60</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1738,22 +1738,22 @@
         <v>20</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>16</v>
@@ -1764,22 +1764,22 @@
         <v>21</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>14</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>16</v>
@@ -1790,19 +1790,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="G26" s="12" t="s">
         <v>106</v>
@@ -1884,19 +1884,19 @@
       </c>
       <c r="E31" s="20" t="n">
         <f aca="false">COUNTIFS(B5:B26,"Processo",H5:H26,"Concluído")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F31" s="20" t="n">
         <f aca="false">D31-E31</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G31" s="21" t="n">
         <f aca="false">E31/D31</f>
-        <v>0.285714285714286</v>
+        <v>0.428571428571429</v>
       </c>
       <c r="H31" s="22" t="n">
         <f aca="false">C31*G31</f>
-        <v>0.571428571428571</v>
+        <v>0.857142857142857</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1911,24 +1911,24 @@
       </c>
       <c r="E32" s="20" t="n">
         <f aca="false">COUNTIFS(B5:B26,"Configuração",H5:H26,"Concluído")</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F32" s="20" t="n">
         <f aca="false">D32-E32</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G32" s="21" t="n">
         <f aca="false">E32/D32</f>
-        <v>0.375</v>
+        <v>0.875</v>
       </c>
       <c r="H32" s="22" t="n">
         <f aca="false">C32*G32</f>
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C33" s="19" t="n">
         <v>1</v>
@@ -1967,19 +1967,19 @@
       </c>
       <c r="E34" s="24" t="n">
         <f aca="false">SUM(E30:E33)</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
         <f aca="false">SUM(F30:F33)</f>
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G34" s="25" t="n">
         <f aca="false">E34/D34</f>
-        <v>0.5</v>
+        <v>0.727272727272727</v>
       </c>
       <c r="H34" s="26" t="n">
         <f aca="false">SUM(H30:H33)</f>
-        <v>6.98809523809524</v>
+        <v>8.27380952380952</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,10 +2002,10 @@
     </row>
     <row r="39" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="C39" s="29" t="s">
         <v>117</v>
-      </c>
-      <c r="C39" s="29" t="s">
-        <v>118</v>
       </c>
       <c r="D39" s="29"/>
       <c r="E39" s="29"/>
@@ -2015,10 +2015,10 @@
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C40" s="29" t="s">
         <v>119</v>
-      </c>
-      <c r="C40" s="29" t="s">
-        <v>120</v>
       </c>
       <c r="D40" s="29"/>
       <c r="E40" s="29"/>
@@ -2031,7 +2031,7 @@
         <v>44</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D41" s="29"/>
       <c r="E41" s="29"/>
@@ -2041,10 +2041,10 @@
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="C42" s="29" t="s">
         <v>122</v>
-      </c>
-      <c r="C42" s="29" t="s">
-        <v>123</v>
       </c>
       <c r="D42" s="29"/>
       <c r="E42" s="29"/>
@@ -2054,12 +2054,12 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="32" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C45" s="32"/>
       <c r="D45" s="32"/>
@@ -2070,7 +2070,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C46" s="32"/>
       <c r="D46" s="32"/>
@@ -2081,7 +2081,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C47" s="32"/>
       <c r="D47" s="32"/>
@@ -2092,7 +2092,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C48" s="32"/>
       <c r="D48" s="32"/>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C49" s="32"/>
       <c r="D49" s="32"/>
@@ -2114,7 +2114,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="32" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C50" s="32"/>
       <c r="D50" s="32"/>
@@ -2178,7 +2178,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2189,7 +2189,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2198,110 +2198,100 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E3" s="3" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="B4" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="4" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="33" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="s">
+      <c r="B5" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="9"/>
       <c r="D5" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
         <v>144</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B12" s="35"/>
       <c r="C12" s="35"/>
@@ -2310,7 +2300,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="35" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="35"/>
@@ -2319,40 +2309,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="35" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B14" s="35"/>
       <c r="C14" s="35"/>
       <c r="D14" s="35"/>
       <c r="E14" s="35"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A16:E16"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>